<commit_message>
fix: update feature importance and leaderboard files
</commit_message>
<xml_diff>
--- a/backend/models/tabpfn_adasyn/feature_importance.xlsx
+++ b/backend/models/tabpfn_adasyn/feature_importance.xlsx
@@ -425,36 +425,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>importance</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>stddev</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>p99_high</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>p99_low</t>
         </is>
@@ -462,301 +472,421 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ffr</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>0.03137254901960784</v>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
         <v>0.02601274345376784</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>0.02713700798481922</v>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
         <v>0.08493314732523839</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>-0.02218804928602271</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>plaque_volume_percent</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>0.009411764705882364</v>
       </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
         <v>0.01318253828546796</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>0.0928112270947878</v>
       </c>
-      <c r="D3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.03655479323770277</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>-0.01773126382593804</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>lumen_area</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>0.00705882352941174</v>
       </c>
-      <c r="B4" t="n">
+      <c r="D4" t="n">
         <v>0.005113099925649118</v>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>0.01834099470022052</v>
       </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.01758676694687447</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>-0.003469119888050987</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bmi</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>0.00470588235294116</v>
       </c>
-      <c r="B5" t="n">
+      <c r="D5" t="n">
         <v>0.004295863196118935</v>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>0.03524199845510997</v>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.01355112404888927</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>-0.004139359343006945</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>syntax_score</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>0.001568627450980387</v>
       </c>
-      <c r="B6" t="n">
+      <c r="D6" t="n">
         <v>0.002147931598059467</v>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>0.08890390417811055</v>
       </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.005991248298954439</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>-0.002853993396993666</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hypertension</t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>diabetes_mellitus</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>multifocal_atherosclerosis</t>
+        </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>post_infarction_cardiosclerosis</t>
+        </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>angina_functional_class</t>
+        </is>
       </c>
       <c r="C13" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cholesterol_level</t>
+        </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lvef_percent</t>
+        </is>
       </c>
       <c r="C15" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>unstable_plaque</t>
+        </is>
       </c>
       <c r="C16" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Model and UI update (#10)
* fix: update feature importance and leaderboard files

* style: refresh global CSS variables and styles for improved UI consistency and accessibility

* style: update global CSS color variables and component styles

* style: update summary group styles and colors for improved visual distinction

* style: refine global CSS variables and enhance component styles for improved visual hierarchy and accessibility

* style: update muted color variable in global CSS for improved visual consistency
</commit_message>
<xml_diff>
--- a/backend/models/tabpfn_adasyn/feature_importance.xlsx
+++ b/backend/models/tabpfn_adasyn/feature_importance.xlsx
@@ -425,36 +425,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>importance</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>stddev</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>p99_high</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>p99_low</t>
         </is>
@@ -462,301 +472,421 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ffr</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>0.03137254901960784</v>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
         <v>0.02601274345376784</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>0.02713700798481922</v>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
         <v>0.08493314732523839</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>-0.02218804928602271</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>plaque_volume_percent</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>0.009411764705882364</v>
       </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
         <v>0.01318253828546796</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>0.0928112270947878</v>
       </c>
-      <c r="D3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.03655479323770277</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>-0.01773126382593804</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>lumen_area</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>0.00705882352941174</v>
       </c>
-      <c r="B4" t="n">
+      <c r="D4" t="n">
         <v>0.005113099925649118</v>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>0.01834099470022052</v>
       </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.01758676694687447</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>-0.003469119888050987</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bmi</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>0.00470588235294116</v>
       </c>
-      <c r="B5" t="n">
+      <c r="D5" t="n">
         <v>0.004295863196118935</v>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>0.03524199845510997</v>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.01355112404888927</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>-0.004139359343006945</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>syntax_score</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>0.001568627450980387</v>
       </c>
-      <c r="B6" t="n">
+      <c r="D6" t="n">
         <v>0.002147931598059467</v>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>0.08890390417811055</v>
       </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.005991248298954439</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>-0.002853993396993666</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hypertension</t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>diabetes_mellitus</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>multifocal_atherosclerosis</t>
+        </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>post_infarction_cardiosclerosis</t>
+        </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>angina_functional_class</t>
+        </is>
       </c>
       <c r="C13" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cholesterol_level</t>
+        </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lvef_percent</t>
+        </is>
       </c>
       <c r="C15" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>unstable_plaque</t>
+        </is>
       </c>
       <c r="C16" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>